<commit_message>
Research: IBB and XLB study workbooks; ARKQ regenerated with an Overlap vs S&P 500 tab
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kn9FvRUhfk3FShXDYTTURS
</commit_message>
<xml_diff>
--- a/research/index-studies/ARKQ_Weights_PE_Sales.xlsx
+++ b/research/index-studies/ARKQ_Weights_PE_Sales.xlsx
@@ -10,9 +10,10 @@
   <sheets>
     <sheet name="Holdings" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Sectors" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Annual Returns" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="By Decade" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Overlap vs S&amp;P 500" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Annual Returns" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="By Decade" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Holdings!$A$1:$N$38</definedName>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="196">
   <si>
     <t xml:space="preserve">Rank</t>
   </si>
@@ -410,34 +411,61 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
+    <t xml:space="preserve">Holdings shared with the S&amp;P 500 (S&amp;P weights from the companion S&amp;P 500 workbook, Sept 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 of 37 holdings are S&amp;P 500 members</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of this fund's weight that is inside the S&amp;P 500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of the S&amp;P 500 that those names represent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weight in this fund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weight in S&amp;P 500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratio (fund ÷ S&amp;P)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total (shared names)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ARKQ: ARK Autonomous Technology &amp; Robotics ETF, constituents, weights, trailing P/E and fund history</t>
   </si>
   <si>
-    <t xml:space="preserve">Holdings and weights: ARK Investment Management's daily holdings file (ark-funds.com), as of 09/22/2026. The cash line (Goldman treasury fund, ~0.2%) is removed and weights rescaled to 100%. ARKQ is actively managed: this is a manager's portfolio of about 35-40 stocks, not a rules-based index, and holdings change frequently.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P/E (TTM), EPS (TTM), Market Cap, Price/Sales, Price, Company name, GICS sector and Sub-Industry: Yahoo Finance via the yfinance library, retrieved Sept 22, 2026. Yahoo's sectors are mapped to GICS sector names; Yahoo's industry label stands in for the GICS sub-industry. ADR lines (Komatsu, BYD, Baidu, WeRide, Pony) may show blanks where Yahoo mixes a USD price with local-currency earnings.</t>
+    <t xml:space="preserve">Holdings and weights: ARK Investment Management's daily holdings file (ark-funds.com). The cash line (~0.2%) is removed and weights rescaled to 100%. ARKQ is actively managed: a manager's portfolio of about 35-40 stocks, not a rules-based index, and holdings change frequently. As of 09/22/2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/E (TTM), EPS (TTM), Market Cap, Price/Sales, Price, Company name, GICS sector and Sub-Industry: Yahoo Finance via the yfinance library, retrieved Sept 23, 2026. Yahoo's sectors are mapped to GICS sector names; Yahoo's industry label stands in for the GICS sub-industry.</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue TTM ($B) is derived as Market Cap / Price-to-Sales, so it is approximate. Blank where either input is missing.</t>
   </si>
   <si>
-    <t xml:space="preserve">Many ARKQ holdings are pre-profit (eVTOL, space, autonomy start-ups). Where trailing EPS is negative, P/E is left blank; expect far more blanks than in the S&amp;P 500 file. The Sectors tab average excludes blanks and P/Es above 100, and shows blank for a sector with no usable P/E.</t>
+    <t xml:space="preserve">Many ARKQ holdings are pre-profit (eVTOL, space, autonomy start-ups). Where trailing EPS is negative, P/E is left blank; expect far more blanks than in the S&amp;P 500 file. The Sectors tab average excludes blanks and P/Es above 100.</t>
   </si>
   <si>
     <t xml:space="preserve">Cumulative Weight assumes the default sort by rank; after re-sorting it shows the running weight in the new order.</t>
   </si>
   <si>
+    <t xml:space="preserve">Overlap tab: every holding whose ticker also appears in the companion S&amp;P 500 workbook, with its weight in each. 'Ratio' shows how many times more concentrated the name is here than in the index.</t>
+  </si>
+  <si>
     <t xml:space="preserve">For information only; not investment advice.</t>
   </si>
   <si>
-    <t xml:space="preserve">Historical tabs 'Annual Returns' (2015-2025) and 'By Decade': ARKQ launched September 30, 2014, so there is no long history and no index to proxy it with. Returns are the fund's own, from Yahoo Finance daily prices: Price Return uses closing prices on the last trading day of each year; Total Return uses dividend-adjusted closes (distributions reinvested). S&amp;P 500 total return (SPY, dividend-adjusted) is shown alongside for comparison. 2014 is a stub period and is excluded.</t>
+    <t xml:space="preserve">Historical tabs 'Annual Returns' (2015-2025) and 'By Decade': the fund launched September 30, 2014, so returns are the fund's own, from Yahoo Finance daily prices. Price Return uses closing prices on the last trading day of each year; Total Return uses dividend-adjusted closes (distributions reinvested). S&amp;P 500 total return (SPY, dividend-adjusted) is shown alongside for the same years. The launch year is a stub and is excluded; 2026 is incomplete and excluded.</t>
   </si>
   <si>
     <t xml:space="preserve">Real returns use December-over-December US CPI-U (NSA) from the BLS (series CUUR0000SA0).</t>
   </si>
   <si>
-    <t xml:space="preserve">Fees: ARKQ's expense ratio is 0.75%, versus 0.03% to 0.05% for the index funds in the companion workbooks. The fund's returns above are net of that fee.</t>
+    <t xml:space="preserve">Fees: the fund's expense ratio is 0.75%; returns above are net of it. The index funds in the companion workbooks charge 0.03% to 0.05%.</t>
   </si>
   <si>
     <t xml:space="preserve">Year</t>
@@ -519,10 +547,13 @@
     <t xml:space="preserve">S&amp;P 500 (SPY) $1 grew to</t>
   </si>
   <si>
+    <t xml:space="preserve">S&amp;P 500 (SPY) standard deviation</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fund returns from Yahoo Finance daily data (last trading day of each year). Total return reinvests distributions. Real returns are CPI-adjusted. 'Average' is the simple mean; 'Annualized / CAGR' is the compound rate actually earned.</t>
   </si>
   <si>
-    <t xml:space="preserve">2014 (fund launched Sept 30) and 2026 (incomplete) are excluded. See the Notes tab.</t>
+    <t xml:space="preserve">2014 (launch year, partial) and 2026 (incomplete) are excluded. See the Notes tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Years
@@ -601,7 +632,7 @@
     <t xml:space="preserve">2015–2025</t>
   </si>
   <si>
-    <t xml:space="preserve">Both decades are partial: the fund launched Sept 30, 2014 and 2026 is incomplete.</t>
+    <t xml:space="preserve">Decades are calendar decades; partial decades are marked.</t>
   </si>
   <si>
     <t xml:space="preserve">Avg Annual = simple average of the yearly returns. Annualized (CAGR) = the compound rate that turns the starting dollar into the ending dollar.</t>
@@ -614,18 +645,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
     <numFmt numFmtId="168" formatCode="0.00"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
-    <numFmt numFmtId="170" formatCode="0"/>
-    <numFmt numFmtId="171" formatCode="0.00%;[RED]\-0.00%"/>
-    <numFmt numFmtId="172" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="173" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="174" formatCode="\$#,##0"/>
+    <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="0.0\x"/>
+    <numFmt numFmtId="172" formatCode="0"/>
+    <numFmt numFmtId="173" formatCode="0.00%;[RED]\-0.00%"/>
+    <numFmt numFmtId="174" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="175" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="\$#,##0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -673,13 +706,6 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -687,6 +713,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -753,7 +786,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -802,11 +835,35 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -814,31 +871,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -850,11 +895,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3080,10 +3125,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3091,52 +3137,292 @@
         <v>127</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
         <v>129</v>
       </c>
+      <c r="B3" s="14" t="n">
+        <v>0.5489</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="B4" s="15" t="n">
+        <v>0.2567</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="C6" s="1" t="s">
         <v>132</v>
       </c>
+      <c r="D6" s="1" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>133</v>
+      <c r="A7" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>0.1079</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>0.0208</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <f aca="false">IF(C7&gt;0,B7/C7,"")</f>
+        <v>5.1875</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12"/>
-    </row>
-    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A8" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>0.0632</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <f aca="false">IF(C8&gt;0,B8/C8,"")</f>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>0.0498</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>0.0773</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <f aca="false">IF(C9&gt;0,B9/C9,"")</f>
+        <v>0.644243208279431</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>0.0489</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <f aca="false">IF(C10&gt;0,B10/C10,"")</f>
+        <v>3.64925373134328</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>0.0465</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>0.0294</v>
+      </c>
+      <c r="D11" s="17" t="n">
+        <f aca="false">IF(C11&gt;0,B11/C11,"")</f>
+        <v>1.58163265306122</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>0.0464</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>0.0061</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <f aca="false">IF(C12&gt;0,B12/C12,"")</f>
+        <v>7.60655737704918</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>0.0348</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>0.0394</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <f aca="false">IF(C13&gt;0,B13/C13,"")</f>
+        <v>0.883248730964467</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>0.0288</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <f aca="false">IF(C14&gt;0,B14/C14,"")</f>
+        <v>11.0769230769231</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>0.0272</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <f aca="false">IF(C15&gt;0,B15/C15,"")</f>
+        <v>38.8571428571429</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>0.0224</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>0.0247</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <f aca="false">IF(C16&gt;0,B16/C16,"")</f>
+        <v>0.906882591093117</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <f aca="false">IF(C17&gt;0,B17/C17,"")</f>
+        <v>98.5</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <f aca="false">IF(C18&gt;0,B18/C18,"")</f>
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B19" s="16" t="n">
+        <v>0.0135</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <f aca="false">IF(C19&gt;0,B19/C19,"")</f>
+        <v>6.75</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="16" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="D20" s="17" t="n">
+        <f aca="false">IF(C20&gt;0,B20/C20,"")</f>
+        <v>2.48148148148148</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="16" t="n">
+        <v>0.0088</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="D21" s="17" t="n">
+        <f aca="false">IF(C21&gt;0,B21/C21,"")</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="C22" s="16" t="n">
+        <v>0.0316</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <f aca="false">IF(C22&gt;0,B22/C22,"")</f>
+        <v>0.0886075949367089</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>136</v>
+      <c r="B23" s="14" t="n">
+        <f aca="false">SUM(B7:B22)</f>
+        <v>0.5488</v>
+      </c>
+      <c r="C23" s="15" t="n">
+        <f aca="false">SUM(C7:C22)</f>
+        <v>0.2567</v>
       </c>
     </row>
   </sheetData>
@@ -3155,7 +3441,87 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110.04"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18"/>
+    </row>
+    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>145</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3171,562 +3537,571 @@
   <sheetData>
     <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="n">
+      <c r="A2" s="19" t="n">
         <v>2015</v>
       </c>
-      <c r="B2" s="14" t="str">
+      <c r="B2" s="20" t="str">
         <f aca="false">INT(A2/10)*10&amp;"s"</f>
         <v>2010s</v>
       </c>
-      <c r="C2" s="15" t="n">
+      <c r="C2" s="21" t="n">
         <v>-0.0338</v>
       </c>
-      <c r="D2" s="15" t="n">
+      <c r="D2" s="21" t="n">
         <v>-0.0245</v>
       </c>
-      <c r="E2" s="15" t="n">
+      <c r="E2" s="21" t="n">
         <v>-0.0408</v>
       </c>
-      <c r="F2" s="15" t="n">
+      <c r="F2" s="21" t="n">
         <v>-0.0315</v>
       </c>
-      <c r="G2" s="14" t="str">
+      <c r="G2" s="20" t="str">
         <f aca="false">IF(D2&gt;=0,"Up","Down")</f>
         <v>Down</v>
       </c>
-      <c r="H2" s="16" t="n">
+      <c r="H2" s="22" t="n">
         <f aca="false">1+D2</f>
         <v>0.9755</v>
       </c>
-      <c r="I2" s="16" t="n">
+      <c r="I2" s="22" t="n">
         <f aca="false">1+C2</f>
         <v>0.9662</v>
       </c>
-      <c r="J2" s="15" t="n">
+      <c r="J2" s="21" t="n">
         <v>0.0123</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="n">
+      <c r="A3" s="19" t="n">
         <v>2016</v>
       </c>
-      <c r="B3" s="14" t="str">
+      <c r="B3" s="20" t="str">
         <f aca="false">INT(A3/10)*10&amp;"s"</f>
         <v>2010s</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="21" t="n">
         <v>0.1451</v>
       </c>
-      <c r="D3" s="15" t="n">
+      <c r="D3" s="21" t="n">
         <v>0.1451</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="21" t="n">
         <v>0.1218</v>
       </c>
-      <c r="F3" s="15" t="n">
+      <c r="F3" s="21" t="n">
         <v>0.1218</v>
       </c>
-      <c r="G3" s="14" t="str">
+      <c r="G3" s="20" t="str">
         <f aca="false">IF(D3&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H3" s="16" t="n">
+      <c r="H3" s="22" t="n">
         <f aca="false">H2*(1+D3)</f>
         <v>1.11704505</v>
       </c>
-      <c r="I3" s="16" t="n">
+      <c r="I3" s="22" t="n">
         <f aca="false">I2*(1+C3)</f>
         <v>1.10639562</v>
       </c>
-      <c r="J3" s="15" t="n">
+      <c r="J3" s="21" t="n">
         <v>0.12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="n">
+      <c r="A4" s="19" t="n">
         <v>2017</v>
       </c>
-      <c r="B4" s="14" t="str">
+      <c r="B4" s="20" t="str">
         <f aca="false">INT(A4/10)*10&amp;"s"</f>
         <v>2010s</v>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="21" t="n">
         <v>0.4998</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="21" t="n">
         <v>0.5226</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="21" t="n">
         <v>0.4688</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="21" t="n">
         <v>0.4912</v>
       </c>
-      <c r="G4" s="14" t="str">
+      <c r="G4" s="20" t="str">
         <f aca="false">IF(D4&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H4" s="16" t="n">
+      <c r="H4" s="22" t="n">
         <f aca="false">H3*(1+D4)</f>
         <v>1.70081279313</v>
       </c>
-      <c r="I4" s="16" t="n">
+      <c r="I4" s="22" t="n">
         <f aca="false">I3*(1+C4)</f>
         <v>1.659372150876</v>
       </c>
-      <c r="J4" s="15" t="n">
+      <c r="J4" s="21" t="n">
         <v>0.2171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="n">
+      <c r="A5" s="19" t="n">
         <v>2018</v>
       </c>
-      <c r="B5" s="14" t="str">
+      <c r="B5" s="20" t="str">
         <f aca="false">INT(A5/10)*10&amp;"s"</f>
         <v>2010s</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="21" t="n">
         <v>-0.1047</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="21" t="n">
         <v>-0.0789</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="21" t="n">
         <v>-0.1215</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="21" t="n">
         <v>-0.0962</v>
       </c>
-      <c r="G5" s="14" t="str">
+      <c r="G5" s="20" t="str">
         <f aca="false">IF(D5&gt;=0,"Up","Down")</f>
         <v>Down</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="22" t="n">
         <f aca="false">H4*(1+D5)</f>
         <v>1.56661866375204</v>
       </c>
-      <c r="I5" s="16" t="n">
+      <c r="I5" s="22" t="n">
         <f aca="false">I4*(1+C5)</f>
         <v>1.48563588667928</v>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="J5" s="21" t="n">
         <v>-0.0457</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="19" t="n">
         <v>2019</v>
       </c>
-      <c r="B6" s="14" t="str">
+      <c r="B6" s="20" t="str">
         <f aca="false">INT(A6/10)*10&amp;"s"</f>
         <v>2010s</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="21" t="n">
         <v>0.2594</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="21" t="n">
         <v>0.2594</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="21" t="n">
         <v>0.2313</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="21" t="n">
         <v>0.2313</v>
       </c>
-      <c r="G6" s="14" t="str">
+      <c r="G6" s="20" t="str">
         <f aca="false">IF(D6&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="22" t="n">
         <f aca="false">H5*(1+D6)</f>
         <v>1.97299954512932</v>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" s="22" t="n">
         <f aca="false">I5*(1+C6)</f>
         <v>1.87100983568389</v>
       </c>
-      <c r="J6" s="15" t="n">
+      <c r="J6" s="21" t="n">
         <v>0.3122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="19" t="n">
         <v>2020</v>
       </c>
-      <c r="B7" s="14" t="str">
+      <c r="B7" s="20" t="str">
         <f aca="false">INT(A7/10)*10&amp;"s"</f>
         <v>2020s</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="21" t="n">
         <v>1.0541</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="21" t="n">
         <v>1.072</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="21" t="n">
         <v>1.0265</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="21" t="n">
         <v>1.0442</v>
       </c>
-      <c r="G7" s="14" t="str">
+      <c r="G7" s="20" t="str">
         <f aca="false">IF(D7&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="22" t="n">
         <f aca="false">H6*(1+D7)</f>
         <v>4.08805505750796</v>
       </c>
-      <c r="I7" s="16" t="n">
+      <c r="I7" s="22" t="n">
         <f aca="false">I6*(1+C7)</f>
         <v>3.84324130347828</v>
       </c>
-      <c r="J7" s="15" t="n">
+      <c r="J7" s="21" t="n">
         <v>0.1833</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="19" t="n">
         <v>2021</v>
       </c>
-      <c r="B8" s="14" t="str">
+      <c r="B8" s="20" t="str">
         <f aca="false">INT(A8/10)*10&amp;"s"</f>
         <v>2020s</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="21" t="n">
         <v>0.0094</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="21" t="n">
         <v>0.0174</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="21" t="n">
         <v>-0.0569</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="21" t="n">
         <v>-0.0494</v>
       </c>
-      <c r="G8" s="14" t="str">
+      <c r="G8" s="20" t="str">
         <f aca="false">IF(D8&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="22" t="n">
         <f aca="false">H7*(1+D8)</f>
         <v>4.1591872155086</v>
       </c>
-      <c r="I8" s="16" t="n">
+      <c r="I8" s="22" t="n">
         <f aca="false">I7*(1+C8)</f>
         <v>3.87936777173097</v>
       </c>
-      <c r="J8" s="15" t="n">
+      <c r="J8" s="21" t="n">
         <v>0.2873</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="19" t="n">
         <v>2022</v>
       </c>
-      <c r="B9" s="14" t="str">
+      <c r="B9" s="20" t="str">
         <f aca="false">INT(A9/10)*10&amp;"s"</f>
         <v>2020s</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="21" t="n">
         <v>-0.4675</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="21" t="n">
         <v>-0.4675</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="21" t="n">
         <v>-0.4998</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="21" t="n">
         <v>-0.4998</v>
       </c>
-      <c r="G9" s="14" t="str">
+      <c r="G9" s="20" t="str">
         <f aca="false">IF(D9&gt;=0,"Up","Down")</f>
         <v>Down</v>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="H9" s="22" t="n">
         <f aca="false">H8*(1+D9)</f>
         <v>2.21476719225833</v>
       </c>
-      <c r="I9" s="16" t="n">
+      <c r="I9" s="22" t="n">
         <f aca="false">I8*(1+C9)</f>
         <v>2.06576333844674</v>
       </c>
-      <c r="J9" s="15" t="n">
+      <c r="J9" s="21" t="n">
         <v>-0.1818</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="19" t="n">
         <v>2023</v>
       </c>
-      <c r="B10" s="14" t="str">
+      <c r="B10" s="20" t="str">
         <f aca="false">INT(A10/10)*10&amp;"s"</f>
         <v>2020s</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="21" t="n">
         <v>0.407</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="21" t="n">
         <v>0.407</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="21" t="n">
         <v>0.3613</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="21" t="n">
         <v>0.3613</v>
       </c>
-      <c r="G10" s="14" t="str">
+      <c r="G10" s="20" t="str">
         <f aca="false">IF(D10&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H10" s="16" t="n">
+      <c r="H10" s="22" t="n">
         <f aca="false">H9*(1+D10)</f>
         <v>3.11617743950747</v>
       </c>
-      <c r="I10" s="16" t="n">
+      <c r="I10" s="22" t="n">
         <f aca="false">I9*(1+C10)</f>
         <v>2.90652901719457</v>
       </c>
-      <c r="J10" s="15" t="n">
+      <c r="J10" s="21" t="n">
         <v>0.2618</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="19" t="n">
         <v>2024</v>
       </c>
-      <c r="B11" s="14" t="str">
+      <c r="B11" s="20" t="str">
         <f aca="false">INT(A11/10)*10&amp;"s"</f>
         <v>2020s</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="21" t="n">
         <v>0.3388</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="21" t="n">
         <v>0.3388</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="21" t="n">
         <v>0.3012</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="21" t="n">
         <v>0.3012</v>
       </c>
-      <c r="G11" s="14" t="str">
+      <c r="G11" s="20" t="str">
         <f aca="false">IF(D11&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="22" t="n">
         <f aca="false">H10*(1+D11)</f>
         <v>4.1719383560126</v>
       </c>
-      <c r="I11" s="16" t="n">
+      <c r="I11" s="22" t="n">
         <f aca="false">I10*(1+C11)</f>
         <v>3.89126104822009</v>
       </c>
-      <c r="J11" s="15" t="n">
+      <c r="J11" s="21" t="n">
         <v>0.2489</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="19" t="n">
         <v>2025</v>
       </c>
-      <c r="B12" s="14" t="str">
+      <c r="B12" s="20" t="str">
         <f aca="false">INT(A12/10)*10&amp;"s"</f>
         <v>2020s</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="21" t="n">
         <v>0.4843</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="21" t="n">
         <v>0.4881</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="21" t="n">
         <v>0.4456</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="21" t="n">
         <v>0.4493</v>
       </c>
-      <c r="G12" s="14" t="str">
+      <c r="G12" s="20" t="str">
         <f aca="false">IF(D12&gt;=0,"Up","Down")</f>
         <v>Up</v>
       </c>
-      <c r="H12" s="16" t="n">
+      <c r="H12" s="22" t="n">
         <f aca="false">H11*(1+D12)</f>
         <v>6.20826146758235</v>
       </c>
-      <c r="I12" s="16" t="n">
+      <c r="I12" s="22" t="n">
         <f aca="false">I11*(1+C12)</f>
         <v>5.77579877387307</v>
       </c>
-      <c r="J12" s="15" t="n">
+      <c r="J12" s="21" t="n">
         <v>0.1772</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
-        <v>147</v>
+      <c r="A14" s="12" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="C15" s="19" t="n">
+      <c r="A15" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="C15" s="23" t="n">
         <f aca="false">COUNT(A2:A12)</f>
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
-        <v>149</v>
-      </c>
-      <c r="C16" s="19" t="n">
+      <c r="A16" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="C16" s="23" t="n">
         <f aca="false">COUNTIF(D2:D12,"&gt;=0")</f>
         <v>8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="C17" s="19" t="n">
+      <c r="A17" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="C17" s="23" t="n">
         <f aca="false">COUNTIF(D2:D12,"&lt;0")</f>
         <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="C18" s="20" t="n">
+      <c r="A18" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="C18" s="16" t="n">
         <f aca="false">AVERAGE(D2:D12)</f>
         <v>0.243590909090909</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="C19" s="20" t="n">
+      <c r="A19" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C19" s="16" t="n">
         <f aca="false">(H12)^(1/COUNT(A2:A12))-1</f>
         <v>0.180560319388258</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="C20" s="20" t="n">
+      <c r="A20" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="C20" s="16" t="n">
         <f aca="false">AVERAGE(F2:F12)</f>
         <v>0.211218181818182</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="C21" s="20" t="n">
+      <c r="A21" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="C21" s="16" t="n">
         <f aca="false">MAX(D2:D12)</f>
         <v>1.072</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
-        <v>155</v>
-      </c>
-      <c r="C22" s="20" t="n">
+      <c r="A22" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="C22" s="16" t="n">
         <f aca="false">MIN(D2:D12)</f>
         <v>-0.4675</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="C23" s="20" t="n">
+      <c r="A23" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" s="16" t="n">
         <f aca="false">STDEV(D2:D12)</f>
         <v>0.400286873266025</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="C24" s="21" t="n">
+      <c r="A24" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="C24" s="24" t="n">
         <f aca="false">H12</f>
         <v>6.20826146758235</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="C25" s="20" t="n">
+      <c r="A25" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="C25" s="16" t="n">
         <f aca="false">AVERAGE(J2:J12)</f>
         <v>0.144781818181818</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="C26" s="20" t="n">
+      <c r="A26" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="C26" s="16" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+J2:J12)))^(1/COUNT(J2:J12))-1</f>
         <v>0.134189306240105</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="C27" s="21" t="n">
+      <c r="A27" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C27" s="24" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+J2:J12)))</f>
         <v>3.9952230462895</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="22" t="s">
-        <v>161</v>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="C28" s="16" t="n">
+        <f aca="false">STDEV(J2:J12)</f>
+        <v>0.155480936568969</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="22" t="s">
-        <v>162</v>
+      <c r="A30" s="25" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="25" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -3740,7 +4115,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3764,244 +4139,244 @@
   <sheetData>
     <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="C2" s="14" t="n">
+      <c r="A2" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C2" s="20" t="n">
         <f aca="false">COUNTIF('Annual Returns'!$B$2:$B$12,"2010s")</f>
         <v>5</v>
       </c>
-      <c r="D2" s="14" t="n">
+      <c r="D2" s="20" t="n">
         <f aca="false">COUNTIFS('Annual Returns'!$B$2:$B$12,"2010s",'Annual Returns'!$D$2:$D$12,"&gt;=0")</f>
         <v>3</v>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="20" t="n">
         <f aca="false">COUNTIFS('Annual Returns'!$B$2:$B$12,"2010s",'Annual Returns'!$D$2:$D$12,"&lt;0")</f>
         <v>2</v>
       </c>
-      <c r="F2" s="15" t="n">
+      <c r="F2" s="21" t="n">
         <f aca="false">AVERAGEIF('Annual Returns'!$B$2:$B$12,"2010s",'Annual Returns'!$D$2:$D$12)</f>
         <v>0.16474</v>
       </c>
-      <c r="G2" s="15" t="n">
+      <c r="G2" s="21" t="n">
         <f aca="false">(1+H2)^(1/C2)-1</f>
         <v>0.145579931640096</v>
       </c>
-      <c r="H2" s="15" t="n">
+      <c r="H2" s="21" t="n">
         <f aca="false">EXP(SUMPRODUCT(('Annual Returns'!$B$2:$B$12="2010s")*LN(1+'Annual Returns'!$D$2:$D$12)))-1</f>
         <v>0.972999545129323</v>
       </c>
-      <c r="I2" s="15" t="n">
+      <c r="I2" s="21" t="n">
         <f aca="false">AVERAGEIF('Annual Returns'!$B$2:$B$12,"2010s",'Annual Returns'!$C$2:$C$12)</f>
         <v>0.15316</v>
       </c>
-      <c r="J2" s="15" t="n">
+      <c r="J2" s="21" t="n">
         <f aca="false">(EXP(SUMPRODUCT(('Annual Returns'!$B$2:$B$12="2010s")*LN(1+'Annual Returns'!$C$2:$C$12))))^(1/C2)-1</f>
         <v>0.13348353022041</v>
       </c>
-      <c r="K2" s="15" t="n">
+      <c r="K2" s="21" t="n">
         <f aca="false">AVERAGEIF('Annual Returns'!$B$2:$B$12,"2010s",'Annual Returns'!$F$2:$F$12)</f>
         <v>0.14332</v>
       </c>
-      <c r="L2" s="15" t="n">
+      <c r="L2" s="21" t="n">
         <f aca="false">_xlfn.MAXIFS('Annual Returns'!$D$2:$D$12,'Annual Returns'!$B$2:$B$12,"2010s")</f>
         <v>0.5226</v>
       </c>
-      <c r="M2" s="15" t="n">
+      <c r="M2" s="21" t="n">
         <f aca="false">_xlfn.MINIFS('Annual Returns'!$D$2:$D$12,'Annual Returns'!$B$2:$B$12,"2010s")</f>
         <v>-0.0789</v>
       </c>
-      <c r="N2" s="16" t="n">
+      <c r="N2" s="22" t="n">
         <f aca="false">1+H2</f>
         <v>1.97299954512932</v>
       </c>
-      <c r="O2" s="15" t="n">
+      <c r="O2" s="21" t="n">
         <f aca="false">(EXP(SUMPRODUCT(('Annual Returns'!$B$2:$B$12="2010s")*LN(1+'Annual Returns'!$J$2:$J$12))))^(1/C2)-1</f>
         <v>0.115597919930413</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="C3" s="14" t="n">
+      <c r="A3" s="20" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="20" t="n">
         <f aca="false">COUNTIF('Annual Returns'!$B$2:$B$12,"2020s")</f>
         <v>6</v>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="D3" s="20" t="n">
         <f aca="false">COUNTIFS('Annual Returns'!$B$2:$B$12,"2020s",'Annual Returns'!$D$2:$D$12,"&gt;=0")</f>
         <v>5</v>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="20" t="n">
         <f aca="false">COUNTIFS('Annual Returns'!$B$2:$B$12,"2020s",'Annual Returns'!$D$2:$D$12,"&lt;0")</f>
         <v>1</v>
       </c>
-      <c r="F3" s="15" t="n">
+      <c r="F3" s="21" t="n">
         <f aca="false">AVERAGEIF('Annual Returns'!$B$2:$B$12,"2020s",'Annual Returns'!$D$2:$D$12)</f>
         <v>0.3093</v>
       </c>
-      <c r="G3" s="15" t="n">
+      <c r="G3" s="21" t="n">
         <f aca="false">(1+H3)^(1/C3)-1</f>
         <v>0.210525202664656</v>
       </c>
-      <c r="H3" s="15" t="n">
+      <c r="H3" s="21" t="n">
         <f aca="false">EXP(SUMPRODUCT(('Annual Returns'!$B$2:$B$12="2020s")*LN(1+'Annual Returns'!$D$2:$D$12)))-1</f>
         <v>2.14661069380805</v>
       </c>
-      <c r="I3" s="15" t="n">
+      <c r="I3" s="21" t="n">
         <f aca="false">AVERAGEIF('Annual Returns'!$B$2:$B$12,"2020s",'Annual Returns'!$C$2:$C$12)</f>
         <v>0.30435</v>
       </c>
-      <c r="J3" s="15" t="n">
+      <c r="J3" s="21" t="n">
         <f aca="false">(EXP(SUMPRODUCT(('Annual Returns'!$B$2:$B$12="2020s")*LN(1+'Annual Returns'!$C$2:$C$12))))^(1/C3)-1</f>
         <v>0.206672264699319</v>
       </c>
-      <c r="K3" s="15" t="n">
+      <c r="K3" s="21" t="n">
         <f aca="false">AVERAGEIF('Annual Returns'!$B$2:$B$12,"2020s",'Annual Returns'!$F$2:$F$12)</f>
         <v>0.2678</v>
       </c>
-      <c r="L3" s="15" t="n">
+      <c r="L3" s="21" t="n">
         <f aca="false">_xlfn.MAXIFS('Annual Returns'!$D$2:$D$12,'Annual Returns'!$B$2:$B$12,"2020s")</f>
         <v>1.072</v>
       </c>
-      <c r="M3" s="15" t="n">
+      <c r="M3" s="21" t="n">
         <f aca="false">_xlfn.MINIFS('Annual Returns'!$D$2:$D$12,'Annual Returns'!$B$2:$B$12,"2020s")</f>
         <v>-0.4675</v>
       </c>
-      <c r="N3" s="16" t="n">
+      <c r="N3" s="22" t="n">
         <f aca="false">1+H3</f>
         <v>3.14661069380805</v>
       </c>
-      <c r="O3" s="15" t="n">
+      <c r="O3" s="21" t="n">
         <f aca="false">(EXP(SUMPRODUCT(('Annual Returns'!$B$2:$B$12="2020s")*LN(1+'Annual Returns'!$J$2:$J$12))))^(1/C3)-1</f>
         <v>0.149918581650387</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
-        <v>181</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="C4" s="23" t="n">
+      <c r="A4" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="C4" s="26" t="n">
         <f aca="false">COUNT('Annual Returns'!$A$2:$A$12)</f>
         <v>11</v>
       </c>
-      <c r="D4" s="23" t="n">
+      <c r="D4" s="26" t="n">
         <f aca="false">COUNTIF('Annual Returns'!$D$2:$D$12,"&gt;=0")</f>
         <v>8</v>
       </c>
-      <c r="E4" s="23" t="n">
+      <c r="E4" s="26" t="n">
         <f aca="false">COUNTIF('Annual Returns'!$D$2:$D$12,"&lt;0")</f>
         <v>3</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="27" t="n">
         <f aca="false">AVERAGE('Annual Returns'!$D$2:$D$12)</f>
         <v>0.243590909090909</v>
       </c>
-      <c r="G4" s="24" t="n">
+      <c r="G4" s="27" t="n">
         <f aca="false">(1+H4)^(1/C4)-1</f>
         <v>0.180560319388258</v>
       </c>
-      <c r="H4" s="24" t="n">
+      <c r="H4" s="27" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+'Annual Returns'!$D$2:$D$12)))-1</f>
         <v>5.20826146758235</v>
       </c>
-      <c r="I4" s="24" t="n">
+      <c r="I4" s="27" t="n">
         <f aca="false">AVERAGE('Annual Returns'!$C$2:$C$12)</f>
         <v>0.235627272727273</v>
       </c>
-      <c r="J4" s="24" t="n">
+      <c r="J4" s="27" t="n">
         <f aca="false">(EXP(SUMPRODUCT(LN(1+'Annual Returns'!$C$2:$C$12))))^(1/C4)-1</f>
         <v>0.172836462813528</v>
       </c>
-      <c r="K4" s="24" t="n">
+      <c r="K4" s="27" t="n">
         <f aca="false">AVERAGE('Annual Returns'!$F$2:$F$12)</f>
         <v>0.211218181818182</v>
       </c>
-      <c r="L4" s="24" t="n">
+      <c r="L4" s="27" t="n">
         <f aca="false">MAX('Annual Returns'!$D$2:$D$12)</f>
         <v>1.072</v>
       </c>
-      <c r="M4" s="24" t="n">
+      <c r="M4" s="27" t="n">
         <f aca="false">MIN('Annual Returns'!$D$2:$D$12)</f>
         <v>-0.4675</v>
       </c>
-      <c r="N4" s="25" t="n">
+      <c r="N4" s="28" t="n">
         <f aca="false">1+H4</f>
         <v>6.20826146758235</v>
       </c>
-      <c r="O4" s="24" t="n">
+      <c r="O4" s="27" t="n">
         <f aca="false">(EXP(SUMPRODUCT(LN(1+'Annual Returns'!$J$2:$J$12))))^(1/C4)-1</f>
         <v>0.134189306240105</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>183</v>
+      <c r="A7" s="25" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>184</v>
+      <c r="A8" s="25" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>185</v>
+      <c r="A9" s="25" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>